<commit_message>
feat(scraper): update SEC RSS pipeline, compliance ledger evidence, and tests
</commit_message>
<xml_diff>
--- a/dpo_system/operator_ledger.xlsx
+++ b/dpo_system/operator_ledger.xlsx
@@ -1923,7 +1923,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P503"/>
+  <dimension ref="A1:P504"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -41160,6 +41160,84 @@
         </is>
       </c>
       <c r="P503" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>doc-20260825204629962245</t>
+        </is>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>docassemble_cli_test</t>
+        </is>
+      </c>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t>approve</t>
+        </is>
+      </c>
+      <c r="D504" t="n">
+        <v>3</v>
+      </c>
+      <c r="E504" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="F504" t="inlineStr">
+        <is>
+          <t>2026-08-25T20:46:29Z</t>
+        </is>
+      </c>
+      <c r="G504" t="inlineStr">
+        <is>
+          <t>2026-08-25T20:46:29Z</t>
+        </is>
+      </c>
+      <c r="H504" t="inlineStr">
+        <is>
+          <t>DPO</t>
+        </is>
+      </c>
+      <c r="I504" t="inlineStr">
+        <is>
+          <t>docassemble-doc-20260825204629962245</t>
+        </is>
+      </c>
+      <c r="J504" t="inlineStr">
+        <is>
+          <t>dpo-system</t>
+        </is>
+      </c>
+      <c r="K504" t="n">
+        <v>1</v>
+      </c>
+      <c r="L504" t="inlineStr">
+        <is>
+          <t>{"crm_action": "classify", "db_table": "casework_employment", "lane": "employment", "taxonomy_key": "us:employment", "template_name": "employment_notice_v1"}</t>
+        </is>
+      </c>
+      <c r="M504" t="inlineStr">
+        <is>
+          <t>employment_launch</t>
+        </is>
+      </c>
+      <c r="N504" t="inlineStr">
+        <is>
+          <t>onboarding</t>
+        </is>
+      </c>
+      <c r="O504" t="inlineStr">
+        <is>
+          <t>docassemble_cli</t>
+        </is>
+      </c>
+      <c r="P504" t="inlineStr">
         <is>
           <t>pending</t>
         </is>

</xml_diff>